<commit_message>
looking at similarity of clipped spectra to sigs
</commit_message>
<xml_diff>
--- a/msi_study/Del2U1_in_fmh_and_pcawg.xlsx
+++ b/msi_study/Del2U1_in_fmh_and_pcawg.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -202,48 +202,52 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -366,15 +370,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>575280</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47520</xdr:rowOff>
+      <xdr:colOff>523800</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>179280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>759240</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>142920</xdr:rowOff>
+      <xdr:colOff>707760</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>84240</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -383,7 +387,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="3051720" y="1952640"/>
+          <a:off x="3000240" y="2274840"/>
           <a:ext cx="798120" cy="4857840"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -575,15 +579,15 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>444960</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>39600</xdr:rowOff>
+      <xdr:colOff>457920</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>105480</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>604440</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>174600</xdr:rowOff>
+      <xdr:colOff>617400</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>50040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -592,7 +596,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="4572360" y="2135160"/>
+          <a:off x="4585320" y="2391480"/>
           <a:ext cx="1458000" cy="1087560"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -800,608 +804,608 @@
   <dimension ref="A1:J44"/>
   <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>46077</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>9.245</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>1.971</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>8951443</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>4765699</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>4185744</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="J5" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>7.833</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>2.16</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>1292986</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>1050186</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>242800</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>6.093</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>2.238</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>428273</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>404726</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="1" t="n">
         <v>23547</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>6.076</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>2.5</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>152728</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>149037</v>
       </c>
-      <c r="G8" s="0" t="n">
+      <c r="G8" s="1" t="n">
         <v>3691</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>11.464</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>1.404</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>880071</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>69015</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="1" t="n">
         <v>811056</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="6" t="n">
         <f aca="false">E9/E5</f>
         <v>0.0983161038952044</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="6" t="n">
         <f aca="false">F9/E5</f>
         <v>0.00770993011964663</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <f aca="false">G9/E5</f>
         <v>0.0906061737755578</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7" t="n">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="8" t="n">
         <f aca="false">E9/(E5+E6+E7+E8)</f>
         <v>0.0812966320968313</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="8" t="n">
         <f aca="false">F9/(E5+E6+E7+E8)</f>
         <v>0.006375266386647</v>
       </c>
-      <c r="G12" s="7" t="n">
+      <c r="G12" s="8" t="n">
         <f aca="false">G9/(E5+E6+E7+E8)</f>
         <v>0.0749213657101843</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>7.465</v>
       </c>
-      <c r="C17" s="0" t="n">
+      <c r="C17" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D17" s="0" t="n">
+      <c r="D17" s="1" t="n">
         <v>1.613</v>
       </c>
-      <c r="E17" s="0" t="n">
+      <c r="E17" s="1" t="n">
         <v>230826</v>
       </c>
-      <c r="F17" s="0" t="n">
+      <c r="F17" s="1" t="n">
         <v>225809</v>
       </c>
-      <c r="G17" s="0" t="n">
+      <c r="G17" s="1" t="n">
         <v>5017</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>6.908</v>
       </c>
-      <c r="C18" s="0" t="n">
+      <c r="C18" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D18" s="0" t="n">
+      <c r="D18" s="1" t="n">
         <v>1.722</v>
       </c>
-      <c r="E18" s="0" t="n">
+      <c r="E18" s="1" t="n">
         <v>121063</v>
       </c>
-      <c r="F18" s="0" t="n">
+      <c r="F18" s="1" t="n">
         <v>119758</v>
       </c>
-      <c r="G18" s="0" t="n">
+      <c r="G18" s="1" t="n">
         <v>1305</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <v>5.248</v>
       </c>
-      <c r="C19" s="0" t="n">
+      <c r="C19" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D19" s="0" t="n">
+      <c r="D19" s="1" t="n">
         <v>1.942</v>
       </c>
-      <c r="E19" s="0" t="n">
+      <c r="E19" s="1" t="n">
         <v>17401</v>
       </c>
-      <c r="F19" s="0" t="n">
+      <c r="F19" s="1" t="n">
         <v>17360</v>
       </c>
-      <c r="G19" s="0" t="n">
+      <c r="G19" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="I19" s="8" t="s">
+      <c r="I19" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <v>4.283</v>
       </c>
-      <c r="C20" s="0" t="n">
+      <c r="C20" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="0" t="n">
+      <c r="D20" s="1" t="n">
         <v>2.894</v>
       </c>
-      <c r="E20" s="0" t="n">
+      <c r="E20" s="1" t="n">
         <v>11071</v>
       </c>
-      <c r="F20" s="0" t="n">
+      <c r="F20" s="1" t="n">
         <v>11067</v>
       </c>
-      <c r="G20" s="0" t="n">
+      <c r="G20" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="I20" s="8"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>9.578</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D21" s="0" t="n">
+      <c r="D21" s="1" t="n">
         <v>1.706</v>
       </c>
-      <c r="E21" s="0" t="n">
+      <c r="E21" s="1" t="n">
         <v>3417</v>
       </c>
-      <c r="F21" s="0" t="n">
+      <c r="F21" s="1" t="n">
         <v>2120</v>
       </c>
-      <c r="G21" s="0" t="n">
+      <c r="G21" s="1" t="n">
         <v>1297</v>
       </c>
-      <c r="I21" s="8"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I22" s="8"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="6" t="n">
         <f aca="false">E21/E17</f>
         <v>0.01480335837384</v>
       </c>
-      <c r="F23" s="5" t="n">
+      <c r="F23" s="6" t="n">
         <f aca="false">F21/E17</f>
         <v>0.00918440730247026</v>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="G23" s="6" t="n">
         <f aca="false">G21/E17</f>
         <v>0.00561895107136978</v>
       </c>
-      <c r="I23" s="8"/>
+      <c r="I23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="7" t="n">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="8" t="n">
         <f aca="false">E21/(E17+E18+E19+E20)</f>
         <v>0.00898357087083061</v>
       </c>
-      <c r="F24" s="7" t="n">
+      <c r="F24" s="8" t="n">
         <f aca="false">F21/(E17+E18+E19+E20)</f>
         <v>0.00557365239864234</v>
       </c>
-      <c r="G24" s="7" t="n">
+      <c r="G24" s="8" t="n">
         <f aca="false">G21/(E17+E18+E19+E20)</f>
         <v>0.00340991847218826</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B29" s="0" t="n">
+      <c r="B29" s="1" t="n">
         <v>7.53</v>
       </c>
-      <c r="C29" s="0" t="n">
+      <c r="C29" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D29" s="0" t="n">
+      <c r="D29" s="1" t="n">
         <v>1.533</v>
       </c>
-      <c r="E29" s="0" t="n">
+      <c r="E29" s="1" t="n">
         <v>788048</v>
       </c>
-      <c r="F29" s="0" t="n">
+      <c r="F29" s="1" t="n">
         <v>770155</v>
       </c>
-      <c r="G29" s="0" t="n">
+      <c r="G29" s="1" t="n">
         <v>17893</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="0" t="n">
+      <c r="B30" s="1" t="n">
         <v>7.046</v>
       </c>
-      <c r="C30" s="0" t="n">
+      <c r="C30" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D30" s="0" t="n">
+      <c r="D30" s="1" t="n">
         <v>1.611</v>
       </c>
-      <c r="E30" s="0" t="n">
+      <c r="E30" s="1" t="n">
         <v>219350</v>
       </c>
-      <c r="F30" s="0" t="n">
+      <c r="F30" s="1" t="n">
         <v>216851</v>
       </c>
-      <c r="G30" s="0" t="n">
+      <c r="G30" s="1" t="n">
         <v>2499</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="0" t="n">
+      <c r="B31" s="1" t="n">
         <v>5.771</v>
       </c>
-      <c r="C31" s="0" t="n">
+      <c r="C31" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D31" s="0" t="n">
+      <c r="D31" s="1" t="n">
         <v>1.546</v>
       </c>
-      <c r="E31" s="0" t="n">
+      <c r="E31" s="1" t="n">
         <v>56690</v>
       </c>
-      <c r="F31" s="0" t="n">
+      <c r="F31" s="1" t="n">
         <v>56569</v>
       </c>
-      <c r="G31" s="0" t="n">
+      <c r="G31" s="1" t="n">
         <v>121</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="0" t="n">
+      <c r="B32" s="1" t="n">
         <v>5.635</v>
       </c>
-      <c r="C32" s="0" t="n">
+      <c r="C32" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D32" s="0" t="n">
+      <c r="D32" s="1" t="n">
         <v>2.029</v>
       </c>
-      <c r="E32" s="0" t="n">
+      <c r="E32" s="1" t="n">
         <v>17208</v>
       </c>
-      <c r="F32" s="0" t="n">
+      <c r="F32" s="1" t="n">
         <v>17205</v>
       </c>
-      <c r="G32" s="0" t="n">
+      <c r="G32" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="1" t="n">
         <v>9.627</v>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="D33" s="0" t="n">
+      <c r="D33" s="1" t="n">
         <v>1.701</v>
       </c>
-      <c r="E33" s="0" t="n">
+      <c r="E33" s="1" t="n">
         <v>12369</v>
       </c>
-      <c r="F33" s="0" t="n">
+      <c r="F33" s="1" t="n">
         <v>7741</v>
       </c>
-      <c r="G33" s="0" t="n">
+      <c r="G33" s="1" t="n">
         <v>4628</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="6" t="n">
         <f aca="false">E33/E29</f>
         <v>0.0156957444216596</v>
       </c>
-      <c r="F35" s="5" t="n">
+      <c r="F35" s="6" t="n">
         <f aca="false">F33/E29</f>
         <v>0.00982300570523623</v>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="6" t="n">
         <f aca="false">G33/E29</f>
         <v>0.00587273871642337</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="7" t="n">
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="8" t="n">
         <f aca="false">E33/(E29+E30+E31+E32)</f>
         <v>0.0114390509166778</v>
       </c>
-      <c r="F36" s="7" t="n">
+      <c r="F36" s="8" t="n">
         <f aca="false">F33/(E29+E30+E31+E32)</f>
         <v>0.00715900179044406</v>
       </c>
-      <c r="G36" s="7" t="n">
+      <c r="G36" s="8" t="n">
         <f aca="false">G33/(E29+E30+E31+E32)</f>
         <v>0.00428004912623371</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H39" s="8" t="s">
+      <c r="H39" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E40" s="9"/>
-      <c r="H40" s="8"/>
-      <c r="J40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="H40" s="9"/>
+      <c r="J40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E41" s="9"/>
-      <c r="H41" s="8"/>
+      <c r="E41" s="10"/>
+      <c r="H41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E42" s="9"/>
-      <c r="H42" s="8"/>
+      <c r="E42" s="10"/>
+      <c r="H42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E43" s="9"/>
-      <c r="H43" s="8"/>
+      <c r="E43" s="10"/>
+      <c r="H43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E44" s="9"/>
+      <c r="E44" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>